<commit_message>
Postive Flow till notice report csv download for flash
</commit_message>
<xml_diff>
--- a/src/test/resources/utilities/TestData.xlsx
+++ b/src/test/resources/utilities/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Backup\Projects\RHB_Project\rhb.com\src\test\resources\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D973ED-21E6-4F83-A644-EEB408B29DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71B0F9B-CD0F-4571-82C1-561E114C7465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="BlockUser" sheetId="3" r:id="rId3"/>
     <sheet name="AccessPermission" sheetId="4" r:id="rId4"/>
     <sheet name="DocSegment" sheetId="5" r:id="rId5"/>
+    <sheet name="Reports" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="61">
   <si>
     <t>Username</t>
   </si>
@@ -172,20 +173,53 @@
     <t>account_number</t>
   </si>
   <si>
-    <t>Groupes</t>
-  </si>
-  <si>
-    <t>Roleses</t>
-  </si>
-  <si>
-    <t>User1112</t>
+    <t>Product Type</t>
+  </si>
+  <si>
+    <t>FromDate</t>
+  </si>
+  <si>
+    <t>ToDate</t>
+  </si>
+  <si>
+    <t>CA Conventional</t>
+  </si>
+  <si>
+    <t>24/FEB/2026</t>
+  </si>
+  <si>
+    <t>Application Name</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>FLASH</t>
+  </si>
+  <si>
+    <t>Current Account</t>
+  </si>
+  <si>
+    <t>ASB</t>
+  </si>
+  <si>
+    <t>AutoGroup</t>
+  </si>
+  <si>
+    <t>AutoRole</t>
+  </si>
+  <si>
+    <t>AutoUser</t>
+  </si>
+  <si>
+    <t>13/NOV/2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,6 +266,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2A00FF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -269,7 +309,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -280,6 +320,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -770,10 +812,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="10"/>
+      <c r="B1" s="12"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
@@ -785,7 +827,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>21</v>
@@ -811,7 +853,7 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>18</v>
@@ -852,7 +894,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>30</v>
@@ -939,4 +981,78 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B7A5B3E-40A8-44FE-B5E9-780A096C58B1}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="15.26953125" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" customWidth="1"/>
+    <col min="4" max="4" width="12.7265625" customWidth="1"/>
+    <col min="5" max="5" width="15.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>